<commit_message>
Clean transit workbook summary presentation
</commit_message>
<xml_diff>
--- a/projects/ntd-michigan-transit/Quincy_Jones_NTD_Transit_Cost_Benchmark.xlsx
+++ b/projects/ntd-michigan-transit/Quincy_Jones_NTD_Transit_Cost_Benchmark.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Summary" sheetId="1" r:id="Rc822df9e445a4f17"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer Analysis" sheetId="2" r:id="Ra9593ea10b47492b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NTD Source" sheetId="3" r:id="Rd3a161fcc52b426e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="R264d52a1d2af4633"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decision Summary" sheetId="1" r:id="R2f7c678388b3491c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Peer Analysis" sheetId="2" r:id="R2119a06d0c364136"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NTD Source" sheetId="3" r:id="R8687adf34e5a4b5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Method" sheetId="4" r:id="R96b110c9a599456a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -23,7 +23,7 @@
     <x:numFmt numFmtId="203" formatCode="#,##0"/>
     <x:numFmt numFmtId="204" formatCode="0.0%"/>
   </x:numFmts>
-  <x:fonts count="8">
+  <x:fonts count="9">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -66,6 +66,11 @@
     <x:font>
       <x:sz val="11"/>
       <x:color rgb="FF17212B"/>
+      <x:name val="Aptos"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Aptos"/>
     </x:font>
   </x:fonts>
@@ -230,7 +235,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="66">
+  <x:cellXfs count="67">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -345,6 +350,7 @@
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
     </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -488,7 +494,7 @@
       </xdr:xfrm>
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R0c1b3ac5766f4a8f"/>
+          <c:chart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" r:id="R68c8fe85d8de43d6"/>
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
@@ -744,10 +750,10 @@
       <x:c r="G2" s="4"/>
       <x:c r="H2" s="4"/>
       <x:c r="I2" s="1"/>
-      <x:c r="J2" s="1" t="str">
+      <x:c r="J2" s="66" t="str">
         <x:v>Agency</x:v>
       </x:c>
-      <x:c r="K2" s="1" t="str">
+      <x:c r="K2" s="66" t="str">
         <x:v>Cost per trip</x:v>
       </x:c>
       <x:c r="L2" s="1"/>
@@ -778,10 +784,10 @@
       <x:c r="G3" s="7"/>
       <x:c r="H3" s="7"/>
       <x:c r="I3" s="1"/>
-      <x:c r="J3" s="1" t="str">
+      <x:c r="J3" s="66" t="str">
         <x:v>University of Michigan Parking and Transportation Services (UMTS) - Logisitics, Transportation &amp; Parking</x:v>
       </x:c>
-      <x:c r="K3" s="1" t="n">
+      <x:c r="K3" s="66" t="n">
         <x:v>2.980545726847554</x:v>
       </x:c>
       <x:c r="L3" s="1"/>
@@ -810,10 +816,10 @@
       <x:c r="G4" s="1"/>
       <x:c r="H4" s="1"/>
       <x:c r="I4" s="1"/>
-      <x:c r="J4" s="1" t="str">
+      <x:c r="J4" s="66" t="str">
         <x:v>Capital Area Transportation Authority (CATA)</x:v>
       </x:c>
-      <x:c r="K4" s="1" t="n">
+      <x:c r="K4" s="66" t="n">
         <x:v>4.480154595441905</x:v>
       </x:c>
       <x:c r="L4" s="1"/>
@@ -848,10 +854,10 @@
       <x:c r="G5" s="17"/>
       <x:c r="H5" s="17"/>
       <x:c r="I5" s="1"/>
-      <x:c r="J5" s="1" t="str">
+      <x:c r="J5" s="66" t="str">
         <x:v>Interurban Transit Partnership (ITP)</x:v>
       </x:c>
-      <x:c r="K5" s="1" t="n">
+      <x:c r="K5" s="66" t="n">
         <x:v>6.481331566966865</x:v>
       </x:c>
       <x:c r="L5" s="1"/>
@@ -895,10 +901,10 @@
         <x:v>First review</x:v>
       </x:c>
       <x:c r="I6" s="1"/>
-      <x:c r="J6" s="1" t="str">
+      <x:c r="J6" s="66" t="str">
         <x:v>Blue Water Area Transportation Commission (BWATC)</x:v>
       </x:c>
-      <x:c r="K6" s="1" t="n">
+      <x:c r="K6" s="66" t="n">
         <x:v>6.58396928935443</x:v>
       </x:c>
       <x:c r="L6" s="1"/>
@@ -942,10 +948,10 @@
         <x:v>Service design / utilization</x:v>
       </x:c>
       <x:c r="I7" s="1"/>
-      <x:c r="J7" s="1" t="str">
+      <x:c r="J7" s="66" t="str">
         <x:v>Mass Transportation Authority (MTA)</x:v>
       </x:c>
-      <x:c r="K7" s="1" t="n">
+      <x:c r="K7" s="66" t="n">
         <x:v>6.957968426348373</x:v>
       </x:c>
       <x:c r="L7" s="1"/>
@@ -989,10 +995,10 @@
         <x:v>Service design / utilization</x:v>
       </x:c>
       <x:c r="I8" s="1"/>
-      <x:c r="J8" s="1" t="str">
+      <x:c r="J8" s="66" t="str">
         <x:v>Central County Transportation Authority (CCTA)</x:v>
       </x:c>
-      <x:c r="K8" s="1" t="n">
+      <x:c r="K8" s="66" t="n">
         <x:v>7.526801567872433</x:v>
       </x:c>
       <x:c r="L8" s="1"/>
@@ -1031,10 +1037,10 @@
         <x:v>Service design / utilization</x:v>
       </x:c>
       <x:c r="I9" s="1"/>
-      <x:c r="J9" s="1" t="str">
+      <x:c r="J9" s="66" t="str">
         <x:v>Ann Arbor Area Transportation Authority (AAATA)</x:v>
       </x:c>
-      <x:c r="K9" s="1" t="n">
+      <x:c r="K9" s="66" t="n">
         <x:v>8.284189069400476</x:v>
       </x:c>
       <x:c r="L9" s="1"/>
@@ -1073,10 +1079,10 @@
         <x:v>Service design / utilization</x:v>
       </x:c>
       <x:c r="I10" s="1"/>
-      <x:c r="J10" s="1" t="str">
+      <x:c r="J10" s="66" t="str">
         <x:v>City of Detroit (DDOT) - Transportation</x:v>
       </x:c>
-      <x:c r="K10" s="1" t="n">
+      <x:c r="K10" s="66" t="n">
         <x:v>8.526353105016002</x:v>
       </x:c>
       <x:c r="L10" s="1"/>
@@ -1115,10 +1121,10 @@
         <x:v>Cost structure / service mix</x:v>
       </x:c>
       <x:c r="I11" s="1"/>
-      <x:c r="J11" s="1" t="str">
+      <x:c r="J11" s="66" t="str">
         <x:v>City of Jackson Transportation Authority (JATA)</x:v>
       </x:c>
-      <x:c r="K11" s="1" t="n">
+      <x:c r="K11" s="66" t="n">
         <x:v>8.812618552308015</x:v>
       </x:c>
       <x:c r="L11" s="1"/>
@@ -1147,10 +1153,10 @@
       <x:c r="G12" s="1"/>
       <x:c r="H12" s="1"/>
       <x:c r="I12" s="1"/>
-      <x:c r="J12" s="1" t="str">
+      <x:c r="J12" s="66" t="str">
         <x:v>Saginaw Transit Authority Regional Service (STARS)</x:v>
       </x:c>
-      <x:c r="K12" s="1" t="n">
+      <x:c r="K12" s="66" t="n">
         <x:v>13.386035647700352</x:v>
       </x:c>
       <x:c r="L12" s="1"/>
@@ -1181,10 +1187,10 @@
       <x:c r="G13" s="17"/>
       <x:c r="H13" s="17"/>
       <x:c r="I13" s="1"/>
-      <x:c r="J13" s="1" t="str">
+      <x:c r="J13" s="66" t="str">
         <x:v>Suburban Mobility Authority for Regional Transportation (SMART)</x:v>
       </x:c>
-      <x:c r="K13" s="1" t="n">
+      <x:c r="K13" s="66" t="n">
         <x:v>14.86440298751742</x:v>
       </x:c>
       <x:c r="L13" s="1"/>
@@ -1215,10 +1221,10 @@
       <x:c r="G14" s="49"/>
       <x:c r="H14" s="50"/>
       <x:c r="I14" s="1"/>
-      <x:c r="J14" s="1" t="str">
+      <x:c r="J14" s="66" t="str">
         <x:v>Lake Erie Transportation Commission (LET) - Operations</x:v>
       </x:c>
-      <x:c r="K14" s="1" t="n">
+      <x:c r="K14" s="66" t="n">
         <x:v>15.061839106654512</x:v>
       </x:c>
       <x:c r="L14" s="1"/>
@@ -1247,10 +1253,10 @@
       <x:c r="G15" s="52"/>
       <x:c r="H15" s="53"/>
       <x:c r="I15" s="1"/>
-      <x:c r="J15" s="1" t="str">
+      <x:c r="J15" s="66" t="str">
         <x:v>Macatawa Area Express Transportation Authority (MAX)</x:v>
       </x:c>
-      <x:c r="K15" s="1" t="n">
+      <x:c r="K15" s="66" t="n">
         <x:v>15.912999619820049</x:v>
       </x:c>
       <x:c r="L15" s="1"/>
@@ -1279,10 +1285,10 @@
       <x:c r="G16" s="52"/>
       <x:c r="H16" s="53"/>
       <x:c r="I16" s="1"/>
-      <x:c r="J16" s="1" t="str">
+      <x:c r="J16" s="66" t="str">
         <x:v>Bay Metropolitan Transit Authority (BMTA)</x:v>
       </x:c>
-      <x:c r="K16" s="1" t="n">
+      <x:c r="K16" s="66" t="n">
         <x:v>20.61079290890974</x:v>
       </x:c>
       <x:c r="L16" s="1"/>
@@ -1311,10 +1317,10 @@
       <x:c r="G17" s="55"/>
       <x:c r="H17" s="56"/>
       <x:c r="I17" s="1"/>
-      <x:c r="J17" s="1" t="str">
+      <x:c r="J17" s="66" t="str">
         <x:v>Bay Area Transportation Authority (BATA)</x:v>
       </x:c>
-      <x:c r="K17" s="1" t="n">
+      <x:c r="K17" s="66" t="n">
         <x:v>26.600895051103382</x:v>
       </x:c>
       <x:c r="L17" s="1"/>
@@ -1343,8 +1349,8 @@
       <x:c r="G18" s="1"/>
       <x:c r="H18" s="1"/>
       <x:c r="I18" s="1"/>
-      <x:c r="J18" s="1"/>
-      <x:c r="K18" s="1"/>
+      <x:c r="J18" s="66"/>
+      <x:c r="K18" s="66"/>
       <x:c r="L18" s="1"/>
       <x:c r="M18" s="1"/>
       <x:c r="N18" s="1"/>
@@ -1373,8 +1379,8 @@
       <x:c r="G19" s="7"/>
       <x:c r="H19" s="7"/>
       <x:c r="I19" s="1"/>
-      <x:c r="J19" s="1"/>
-      <x:c r="K19" s="1"/>
+      <x:c r="J19" s="66"/>
+      <x:c r="K19" s="66"/>
       <x:c r="L19" s="1"/>
       <x:c r="M19" s="1"/>
       <x:c r="N19" s="1"/>
@@ -6469,7 +6475,7 @@
     <x:mergeCell ref="A19:H19"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R33a80a7be1fd4b91"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R578f7d5a603446e1"/>
 </x:worksheet>
 </file>
 

</xml_diff>